<commit_message>
adding model regression of O against final cal results
</commit_message>
<xml_diff>
--- a/cal/cal_results/CS_Ilena_Scattering_Results.xlsx
+++ b/cal/cal_results/CS_Ilena_Scattering_Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonny Woof\Google Drive\Python_packages_woof\pyMAP\cal\cal_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1137102-FD2E-47EB-BBA8-CFE82E540FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378F472D-1A6F-4406-89BC-0F78C3335678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-11550" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cutfit fwhm" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="72">
   <si>
     <t>100A</t>
   </si>
@@ -922,7 +922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:AS246"/>
+  <dimension ref="A2:AS247"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="15.6640625" customWidth="1"/>
@@ -7301,73 +7301,81 @@
       <c r="AI186" s="14"/>
     </row>
     <row r="187" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A187" t="s">
-        <v>41</v>
-      </c>
-      <c r="B187" t="s">
-        <v>64</v>
-      </c>
       <c r="F187">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G187" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H187" t="s">
-        <v>59</v>
-      </c>
-      <c r="I187">
-        <v>1.7</v>
-      </c>
-      <c r="J187">
-        <v>1.7</v>
-      </c>
-      <c r="K187">
-        <v>1.3</v>
-      </c>
-      <c r="L187">
-        <v>1.4</v>
-      </c>
-      <c r="M187">
-        <v>1.9</v>
-      </c>
-      <c r="N187">
-        <v>2.1</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="I187"/>
+      <c r="N187" s="13"/>
       <c r="S187" s="14"/>
       <c r="T187"/>
-      <c r="AF187" s="14"/>
-      <c r="AG187" s="14"/>
+      <c r="U187">
+        <v>0.75529999999999997</v>
+      </c>
+      <c r="V187">
+        <v>0.75760000000000005</v>
+      </c>
+      <c r="W187">
+        <v>0.75219999999999998</v>
+      </c>
+      <c r="X187">
+        <v>0.73640000000000005</v>
+      </c>
+      <c r="Y187">
+        <v>0.74819999999999998</v>
+      </c>
+      <c r="Z187">
+        <v>0.72950000000000004</v>
+      </c>
+      <c r="AA187">
+        <v>0.70709999999999995</v>
+      </c>
       <c r="AI187" s="14"/>
     </row>
     <row r="188" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>41</v>
+      </c>
       <c r="B188" t="s">
         <v>64</v>
       </c>
+      <c r="F188">
+        <v>8</v>
+      </c>
       <c r="G188" t="s">
         <v>3</v>
       </c>
       <c r="H188" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I188">
-        <v>13.7</v>
+        <v>1.7</v>
       </c>
       <c r="J188">
-        <v>14.2</v>
+        <v>1.7</v>
       </c>
       <c r="K188">
-        <v>15</v>
+        <v>1.3</v>
       </c>
       <c r="L188">
-        <v>14.6</v>
+        <v>1.4</v>
       </c>
       <c r="M188">
-        <v>14</v>
+        <v>1.9</v>
       </c>
       <c r="N188">
-        <v>13.8</v>
-      </c>
+        <v>2.1</v>
+      </c>
+      <c r="S188" s="14"/>
+      <c r="T188"/>
+      <c r="AF188" s="14"/>
+      <c r="AG188" s="14"/>
+      <c r="AI188" s="14"/>
     </row>
     <row r="189" spans="1:35" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
@@ -7377,25 +7385,25 @@
         <v>3</v>
       </c>
       <c r="H189" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I189">
-        <v>18.7</v>
+        <v>13.7</v>
       </c>
       <c r="J189">
-        <v>19.600000000000001</v>
+        <v>14.2</v>
       </c>
       <c r="K189">
-        <v>20</v>
-      </c>
-      <c r="L189" t="s">
-        <v>63</v>
-      </c>
-      <c r="M189" t="s">
-        <v>63</v>
-      </c>
-      <c r="N189" t="s">
-        <v>63</v>
+        <v>15</v>
+      </c>
+      <c r="L189">
+        <v>14.6</v>
+      </c>
+      <c r="M189">
+        <v>14</v>
+      </c>
+      <c r="N189">
+        <v>13.8</v>
       </c>
     </row>
     <row r="190" spans="1:35" x14ac:dyDescent="0.3">
@@ -7403,28 +7411,28 @@
         <v>64</v>
       </c>
       <c r="G190" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H190" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I190">
-        <v>1.5</v>
+        <v>18.7</v>
       </c>
       <c r="J190">
-        <v>1.7</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="K190">
-        <v>2</v>
-      </c>
-      <c r="L190">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="M190">
-        <v>2.7</v>
-      </c>
-      <c r="N190">
-        <v>2.2999999999999998</v>
+        <v>20</v>
+      </c>
+      <c r="L190" t="s">
+        <v>63</v>
+      </c>
+      <c r="M190" t="s">
+        <v>63</v>
+      </c>
+      <c r="N190" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="191" spans="1:35" x14ac:dyDescent="0.3">
@@ -7435,25 +7443,25 @@
         <v>4</v>
       </c>
       <c r="H191" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I191">
-        <v>12.7</v>
+        <v>1.5</v>
       </c>
       <c r="J191">
-        <v>11.8</v>
+        <v>1.7</v>
       </c>
       <c r="K191">
-        <v>11.2</v>
+        <v>2</v>
       </c>
       <c r="L191">
-        <v>12</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="M191">
-        <v>12.5</v>
+        <v>2.7</v>
       </c>
       <c r="N191">
-        <v>13</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="192" spans="1:35" x14ac:dyDescent="0.3">
@@ -7464,25 +7472,25 @@
         <v>4</v>
       </c>
       <c r="H192" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I192">
-        <v>16.5</v>
+        <v>12.7</v>
       </c>
       <c r="J192">
-        <v>16.5</v>
+        <v>11.8</v>
       </c>
       <c r="K192">
-        <v>16.600000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="L192">
-        <v>17.8</v>
+        <v>12</v>
       </c>
       <c r="M192">
-        <v>19.2</v>
+        <v>12.5</v>
       </c>
       <c r="N192">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="193" spans="2:14" x14ac:dyDescent="0.3">
@@ -7490,28 +7498,28 @@
         <v>64</v>
       </c>
       <c r="G193" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H193" t="s">
-        <v>59</v>
-      </c>
-      <c r="I193" t="s">
-        <v>9</v>
+        <v>32</v>
+      </c>
+      <c r="I193">
+        <v>16.5</v>
       </c>
       <c r="J193">
-        <v>3.5</v>
+        <v>16.5</v>
       </c>
       <c r="K193">
-        <v>4</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="L193">
-        <v>4.4000000000000004</v>
+        <v>17.8</v>
       </c>
       <c r="M193">
-        <v>4.2</v>
+        <v>19.2</v>
       </c>
       <c r="N193">
-        <v>4.2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="194" spans="2:14" x14ac:dyDescent="0.3">
@@ -7522,25 +7530,25 @@
         <v>6</v>
       </c>
       <c r="H194" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I194" t="s">
         <v>9</v>
       </c>
       <c r="J194">
-        <v>12.9</v>
+        <v>3.5</v>
       </c>
       <c r="K194">
-        <v>12.6</v>
+        <v>4</v>
       </c>
       <c r="L194">
-        <v>13</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="M194">
-        <v>13.2</v>
+        <v>4.2</v>
       </c>
       <c r="N194">
-        <v>13.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="195" spans="2:14" x14ac:dyDescent="0.3">
@@ -7551,25 +7559,25 @@
         <v>6</v>
       </c>
       <c r="H195" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I195" t="s">
         <v>9</v>
       </c>
       <c r="J195">
-        <v>15.5</v>
+        <v>12.9</v>
       </c>
       <c r="K195">
-        <v>15.8</v>
+        <v>12.6</v>
       </c>
       <c r="L195">
-        <v>16.3</v>
+        <v>13</v>
       </c>
       <c r="M195">
-        <v>17.399999999999999</v>
+        <v>13.2</v>
       </c>
       <c r="N195">
-        <v>18</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="196" spans="2:14" x14ac:dyDescent="0.3">
@@ -7577,28 +7585,28 @@
         <v>64</v>
       </c>
       <c r="G196" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H196" t="s">
-        <v>59</v>
-      </c>
-      <c r="I196">
-        <v>8.6999999999999993</v>
+        <v>32</v>
+      </c>
+      <c r="I196" t="s">
+        <v>9</v>
       </c>
       <c r="J196">
-        <v>9.6</v>
+        <v>15.5</v>
       </c>
       <c r="K196">
-        <v>10.8</v>
+        <v>15.8</v>
       </c>
       <c r="L196">
-        <v>11.4</v>
+        <v>16.3</v>
       </c>
       <c r="M196">
-        <v>12.9</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="N196">
-        <v>13.3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="197" spans="2:14" x14ac:dyDescent="0.3">
@@ -7609,25 +7617,25 @@
         <v>5</v>
       </c>
       <c r="H197" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I197">
-        <v>10.3</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="J197">
+        <v>9.6</v>
+      </c>
+      <c r="K197">
         <v>10.8</v>
       </c>
-      <c r="K197">
-        <v>11.6</v>
-      </c>
       <c r="L197">
-        <v>13</v>
+        <v>11.4</v>
       </c>
       <c r="M197">
-        <v>15.3</v>
+        <v>12.9</v>
       </c>
       <c r="N197">
-        <v>16</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="198" spans="2:14" x14ac:dyDescent="0.3">
@@ -7638,54 +7646,54 @@
         <v>5</v>
       </c>
       <c r="H198" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I198">
-        <v>14.4</v>
+        <v>10.3</v>
       </c>
       <c r="J198">
+        <v>10.8</v>
+      </c>
+      <c r="K198">
+        <v>11.6</v>
+      </c>
+      <c r="L198">
+        <v>13</v>
+      </c>
+      <c r="M198">
         <v>15.3</v>
       </c>
-      <c r="K198">
+      <c r="N198">
         <v>16</v>
-      </c>
-      <c r="L198">
-        <v>17.399999999999999</v>
-      </c>
-      <c r="M198">
-        <v>20</v>
-      </c>
-      <c r="N198" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="199" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G199" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H199" t="s">
-        <v>59</v>
-      </c>
-      <c r="I199" t="s">
-        <v>9</v>
-      </c>
-      <c r="J199" t="s">
-        <v>9</v>
+        <v>32</v>
+      </c>
+      <c r="I199">
+        <v>14.4</v>
+      </c>
+      <c r="J199">
+        <v>15.3</v>
       </c>
       <c r="K199">
-        <v>1.9</v>
+        <v>16</v>
       </c>
       <c r="L199">
-        <v>1.6</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="M199">
-        <v>1.9</v>
-      </c>
-      <c r="N199">
-        <v>2.2000000000000002</v>
+        <v>20</v>
+      </c>
+      <c r="N199" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="200" spans="2:14" x14ac:dyDescent="0.3">
@@ -7696,7 +7704,7 @@
         <v>3</v>
       </c>
       <c r="H200" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I200" t="s">
         <v>9</v>
@@ -7705,16 +7713,16 @@
         <v>9</v>
       </c>
       <c r="K200">
-        <v>17</v>
+        <v>1.9</v>
       </c>
       <c r="L200">
-        <v>13.7</v>
+        <v>1.6</v>
       </c>
       <c r="M200">
-        <v>13</v>
+        <v>1.9</v>
       </c>
       <c r="N200">
-        <v>13.4</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="201" spans="2:14" x14ac:dyDescent="0.3">
@@ -7725,7 +7733,7 @@
         <v>3</v>
       </c>
       <c r="H201" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I201" t="s">
         <v>9</v>
@@ -7733,17 +7741,17 @@
       <c r="J201" t="s">
         <v>9</v>
       </c>
-      <c r="K201" t="s">
-        <v>9</v>
-      </c>
-      <c r="L201" t="s">
-        <v>9</v>
-      </c>
-      <c r="M201" t="s">
-        <v>9</v>
-      </c>
-      <c r="N201" t="s">
-        <v>9</v>
+      <c r="K201">
+        <v>17</v>
+      </c>
+      <c r="L201">
+        <v>13.7</v>
+      </c>
+      <c r="M201">
+        <v>13</v>
+      </c>
+      <c r="N201">
+        <v>13.4</v>
       </c>
     </row>
     <row r="202" spans="2:14" x14ac:dyDescent="0.3">
@@ -7751,10 +7759,10 @@
         <v>65</v>
       </c>
       <c r="G202" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H202" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I202" t="s">
         <v>9</v>
@@ -7762,17 +7770,17 @@
       <c r="J202" t="s">
         <v>9</v>
       </c>
-      <c r="K202">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="L202">
-        <v>2.4</v>
-      </c>
-      <c r="M202">
-        <v>2.7</v>
-      </c>
-      <c r="N202">
-        <v>2.7</v>
+      <c r="K202" t="s">
+        <v>9</v>
+      </c>
+      <c r="L202" t="s">
+        <v>9</v>
+      </c>
+      <c r="M202" t="s">
+        <v>9</v>
+      </c>
+      <c r="N202" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="203" spans="2:14" x14ac:dyDescent="0.3">
@@ -7783,7 +7791,7 @@
         <v>4</v>
       </c>
       <c r="H203" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I203" t="s">
         <v>9</v>
@@ -7792,16 +7800,16 @@
         <v>9</v>
       </c>
       <c r="K203">
-        <v>10.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="L203">
-        <v>11.1</v>
+        <v>2.4</v>
       </c>
       <c r="M203">
-        <v>14.5</v>
+        <v>2.7</v>
       </c>
       <c r="N203">
-        <v>12.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="204" spans="2:14" x14ac:dyDescent="0.3">
@@ -7812,7 +7820,7 @@
         <v>4</v>
       </c>
       <c r="H204" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I204" t="s">
         <v>9</v>
@@ -7821,16 +7829,16 @@
         <v>9</v>
       </c>
       <c r="K204">
-        <v>15</v>
+        <v>10.8</v>
       </c>
       <c r="L204">
-        <v>15.5</v>
+        <v>11.1</v>
       </c>
       <c r="M204">
-        <v>21</v>
+        <v>14.5</v>
       </c>
       <c r="N204">
-        <v>19</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="205" spans="2:14" x14ac:dyDescent="0.3">
@@ -7838,10 +7846,10 @@
         <v>65</v>
       </c>
       <c r="G205" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H205" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I205" t="s">
         <v>9</v>
@@ -7850,16 +7858,16 @@
         <v>9</v>
       </c>
       <c r="K205">
-        <v>3.7</v>
+        <v>15</v>
       </c>
       <c r="L205">
-        <v>3.8</v>
+        <v>15.5</v>
       </c>
       <c r="M205">
-        <v>4.0999999999999996</v>
+        <v>21</v>
       </c>
       <c r="N205">
-        <v>4.2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="206" spans="2:14" x14ac:dyDescent="0.3">
@@ -7870,7 +7878,7 @@
         <v>6</v>
       </c>
       <c r="H206" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I206" t="s">
         <v>9</v>
@@ -7879,16 +7887,16 @@
         <v>9</v>
       </c>
       <c r="K206">
-        <v>10.8</v>
+        <v>3.7</v>
       </c>
       <c r="L206">
-        <v>11.1</v>
+        <v>3.8</v>
       </c>
       <c r="M206">
-        <v>11.5</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="N206">
-        <v>12.2</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="207" spans="2:14" x14ac:dyDescent="0.3">
@@ -7899,7 +7907,7 @@
         <v>6</v>
       </c>
       <c r="H207" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I207" t="s">
         <v>9</v>
@@ -7908,16 +7916,16 @@
         <v>9</v>
       </c>
       <c r="K207">
-        <v>14.4</v>
+        <v>10.8</v>
       </c>
       <c r="L207">
-        <v>15</v>
+        <v>11.1</v>
       </c>
       <c r="M207">
-        <v>15.5</v>
+        <v>11.5</v>
       </c>
       <c r="N207">
-        <v>16.8</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="208" spans="2:14" x14ac:dyDescent="0.3">
@@ -7925,10 +7933,10 @@
         <v>65</v>
       </c>
       <c r="G208" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H208" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I208" t="s">
         <v>9</v>
@@ -7937,16 +7945,16 @@
         <v>9</v>
       </c>
       <c r="K208">
-        <v>10.3</v>
+        <v>14.4</v>
       </c>
       <c r="L208">
-        <v>11.6</v>
+        <v>15</v>
       </c>
       <c r="M208">
-        <v>12.3</v>
+        <v>15.5</v>
       </c>
       <c r="N208">
-        <v>12.6</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="209" spans="2:14" x14ac:dyDescent="0.3">
@@ -7957,7 +7965,7 @@
         <v>5</v>
       </c>
       <c r="H209" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I209" t="s">
         <v>9</v>
@@ -7966,16 +7974,16 @@
         <v>9</v>
       </c>
       <c r="K209">
-        <v>11</v>
+        <v>10.3</v>
       </c>
       <c r="L209">
-        <v>12.7</v>
+        <v>11.6</v>
       </c>
       <c r="M209">
-        <v>13.5</v>
+        <v>12.3</v>
       </c>
       <c r="N209">
-        <v>14</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="210" spans="2:14" x14ac:dyDescent="0.3">
@@ -7986,7 +7994,7 @@
         <v>5</v>
       </c>
       <c r="H210" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I210" t="s">
         <v>9</v>
@@ -7995,27 +8003,27 @@
         <v>9</v>
       </c>
       <c r="K210">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="L210">
-        <v>16.2</v>
+        <v>12.7</v>
       </c>
       <c r="M210">
-        <v>18</v>
+        <v>13.5</v>
       </c>
       <c r="N210">
-        <v>19.2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="211" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G211" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H211" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I211" t="s">
         <v>9</v>
@@ -8024,16 +8032,16 @@
         <v>9</v>
       </c>
       <c r="K211">
-        <v>1.3</v>
+        <v>15</v>
       </c>
       <c r="L211">
-        <v>1.8</v>
+        <v>16.2</v>
       </c>
       <c r="M211">
-        <v>1.5</v>
+        <v>18</v>
       </c>
       <c r="N211">
-        <v>2.1</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="212" spans="2:14" x14ac:dyDescent="0.3">
@@ -8044,7 +8052,7 @@
         <v>3</v>
       </c>
       <c r="H212" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I212" t="s">
         <v>9</v>
@@ -8053,16 +8061,16 @@
         <v>9</v>
       </c>
       <c r="K212">
-        <v>15.3</v>
+        <v>1.3</v>
       </c>
       <c r="L212">
-        <v>15</v>
+        <v>1.8</v>
       </c>
       <c r="M212">
-        <v>14.3</v>
+        <v>1.5</v>
       </c>
       <c r="N212">
-        <v>14</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="213" spans="2:14" x14ac:dyDescent="0.3">
@@ -8073,7 +8081,7 @@
         <v>3</v>
       </c>
       <c r="H213" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I213" t="s">
         <v>9</v>
@@ -8082,16 +8090,16 @@
         <v>9</v>
       </c>
       <c r="K213">
-        <v>19.5</v>
+        <v>15.3</v>
       </c>
       <c r="L213">
-        <v>21</v>
-      </c>
-      <c r="M213" t="s">
-        <v>63</v>
-      </c>
-      <c r="N213" t="s">
-        <v>63</v>
+        <v>15</v>
+      </c>
+      <c r="M213">
+        <v>14.3</v>
+      </c>
+      <c r="N213">
+        <v>14</v>
       </c>
     </row>
     <row r="214" spans="2:14" x14ac:dyDescent="0.3">
@@ -8099,10 +8107,10 @@
         <v>66</v>
       </c>
       <c r="G214" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H214" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I214" t="s">
         <v>9</v>
@@ -8111,16 +8119,16 @@
         <v>9</v>
       </c>
       <c r="K214">
-        <v>2.85</v>
+        <v>19.5</v>
       </c>
       <c r="L214">
-        <v>2.4500000000000002</v>
-      </c>
-      <c r="M214">
-        <v>2.9</v>
-      </c>
-      <c r="N214">
-        <v>3.2</v>
+        <v>21</v>
+      </c>
+      <c r="M214" t="s">
+        <v>63</v>
+      </c>
+      <c r="N214" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="215" spans="2:14" x14ac:dyDescent="0.3">
@@ -8131,7 +8139,7 @@
         <v>4</v>
       </c>
       <c r="H215" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I215" t="s">
         <v>9</v>
@@ -8140,16 +8148,16 @@
         <v>9</v>
       </c>
       <c r="K215">
-        <v>12.2</v>
+        <v>2.85</v>
       </c>
       <c r="L215">
-        <v>12.7</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="M215">
-        <v>17.8</v>
+        <v>2.9</v>
       </c>
       <c r="N215">
-        <v>15.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="216" spans="2:14" x14ac:dyDescent="0.3">
@@ -8160,7 +8168,7 @@
         <v>4</v>
       </c>
       <c r="H216" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I216" t="s">
         <v>9</v>
@@ -8169,16 +8177,16 @@
         <v>9</v>
       </c>
       <c r="K216">
-        <v>17.2</v>
+        <v>12.2</v>
       </c>
       <c r="L216">
-        <v>19</v>
+        <v>12.7</v>
       </c>
       <c r="M216">
-        <v>21</v>
-      </c>
-      <c r="N216" t="s">
-        <v>63</v>
+        <v>17.8</v>
+      </c>
+      <c r="N216">
+        <v>15.5</v>
       </c>
     </row>
     <row r="217" spans="2:14" x14ac:dyDescent="0.3">
@@ -8186,10 +8194,10 @@
         <v>66</v>
       </c>
       <c r="G217" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H217" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I217" t="s">
         <v>9</v>
@@ -8198,16 +8206,16 @@
         <v>9</v>
       </c>
       <c r="K217">
-        <v>4.2</v>
+        <v>17.2</v>
       </c>
       <c r="L217">
-        <v>4.3</v>
+        <v>19</v>
       </c>
       <c r="M217">
-        <v>4</v>
-      </c>
-      <c r="N217">
-        <v>4.7</v>
+        <v>21</v>
+      </c>
+      <c r="N217" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="218" spans="2:14" x14ac:dyDescent="0.3">
@@ -8218,7 +8226,7 @@
         <v>6</v>
       </c>
       <c r="H218" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I218" t="s">
         <v>9</v>
@@ -8227,16 +8235,16 @@
         <v>9</v>
       </c>
       <c r="K218">
-        <v>13.1</v>
+        <v>4.2</v>
       </c>
       <c r="L218">
-        <v>13</v>
+        <v>4.3</v>
       </c>
       <c r="M218">
-        <v>13.6</v>
+        <v>4</v>
       </c>
       <c r="N218">
-        <v>14.1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="219" spans="2:14" x14ac:dyDescent="0.3">
@@ -8247,7 +8255,7 @@
         <v>6</v>
       </c>
       <c r="H219" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I219" t="s">
         <v>9</v>
@@ -8256,16 +8264,16 @@
         <v>9</v>
       </c>
       <c r="K219">
-        <v>15.8</v>
+        <v>13.1</v>
       </c>
       <c r="L219">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M219">
-        <v>16.7</v>
+        <v>13.6</v>
       </c>
       <c r="N219">
-        <v>18</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="220" spans="2:14" x14ac:dyDescent="0.3">
@@ -8273,10 +8281,10 @@
         <v>66</v>
       </c>
       <c r="G220" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H220" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I220" t="s">
         <v>9</v>
@@ -8285,16 +8293,16 @@
         <v>9</v>
       </c>
       <c r="K220">
-        <v>11.3</v>
+        <v>15.8</v>
       </c>
       <c r="L220">
-        <v>12.8</v>
+        <v>16</v>
       </c>
       <c r="M220">
-        <v>14.2</v>
+        <v>16.7</v>
       </c>
       <c r="N220">
-        <v>13.9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="221" spans="2:14" x14ac:dyDescent="0.3">
@@ -8305,7 +8313,7 @@
         <v>5</v>
       </c>
       <c r="H221" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I221" t="s">
         <v>9</v>
@@ -8314,16 +8322,16 @@
         <v>9</v>
       </c>
       <c r="K221">
-        <v>12.3</v>
+        <v>11.3</v>
       </c>
       <c r="L221">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="M221">
-        <v>15</v>
+        <v>14.2</v>
       </c>
       <c r="N221">
-        <v>16.2</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="222" spans="2:14" x14ac:dyDescent="0.3">
@@ -8334,7 +8342,7 @@
         <v>5</v>
       </c>
       <c r="H222" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I222" t="s">
         <v>9</v>
@@ -8343,45 +8351,45 @@
         <v>9</v>
       </c>
       <c r="K222">
-        <v>15.6</v>
+        <v>12.3</v>
       </c>
       <c r="L222">
-        <v>15.9</v>
+        <v>13</v>
       </c>
       <c r="M222">
-        <v>19</v>
-      </c>
-      <c r="N222" t="s">
-        <v>63</v>
+        <v>15</v>
+      </c>
+      <c r="N222">
+        <v>16.2</v>
       </c>
     </row>
     <row r="223" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B223" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G223" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H223" t="s">
-        <v>59</v>
-      </c>
-      <c r="I223">
-        <v>1.7</v>
-      </c>
-      <c r="J223">
-        <v>1.7</v>
+        <v>32</v>
+      </c>
+      <c r="I223" t="s">
+        <v>9</v>
+      </c>
+      <c r="J223" t="s">
+        <v>9</v>
       </c>
       <c r="K223">
-        <v>1.3</v>
+        <v>15.6</v>
       </c>
       <c r="L223">
-        <v>1.4</v>
+        <v>15.9</v>
       </c>
       <c r="M223">
-        <v>1.9</v>
-      </c>
-      <c r="N223">
-        <v>2.1</v>
+        <v>19</v>
+      </c>
+      <c r="N223" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="224" spans="2:14" x14ac:dyDescent="0.3">
@@ -8392,25 +8400,25 @@
         <v>3</v>
       </c>
       <c r="H224" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I224">
-        <v>14.5</v>
+        <v>1.7</v>
       </c>
       <c r="J224">
-        <v>16.8</v>
+        <v>1.7</v>
       </c>
       <c r="K224">
-        <v>15.7</v>
+        <v>1.3</v>
       </c>
       <c r="L224">
-        <v>15</v>
+        <v>1.4</v>
       </c>
       <c r="M224">
-        <v>14.7</v>
+        <v>1.9</v>
       </c>
       <c r="N224">
-        <v>15</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="225" spans="2:14" x14ac:dyDescent="0.3">
@@ -8421,25 +8429,25 @@
         <v>3</v>
       </c>
       <c r="H225" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I225">
-        <v>19.5</v>
+        <v>14.5</v>
       </c>
       <c r="J225">
-        <v>21</v>
+        <v>16.8</v>
       </c>
       <c r="K225">
-        <v>21.7</v>
+        <v>15.7</v>
       </c>
       <c r="L225">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="M225">
-        <v>22.7</v>
+        <v>14.7</v>
       </c>
       <c r="N225">
-        <v>23.3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" spans="2:14" x14ac:dyDescent="0.3">
@@ -8447,28 +8455,28 @@
         <v>67</v>
       </c>
       <c r="G226" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H226" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I226">
-        <v>2.2999999999999998</v>
+        <v>19.5</v>
       </c>
       <c r="J226">
-        <v>2.5</v>
+        <v>21</v>
       </c>
       <c r="K226">
-        <v>2.9</v>
+        <v>21.7</v>
       </c>
       <c r="L226">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="M226">
-        <v>3</v>
+        <v>22.7</v>
       </c>
       <c r="N226">
-        <v>3</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="227" spans="2:14" x14ac:dyDescent="0.3">
@@ -8479,25 +8487,25 @@
         <v>4</v>
       </c>
       <c r="H227" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I227">
-        <v>14</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="J227">
-        <v>13.7</v>
+        <v>2.5</v>
       </c>
       <c r="K227">
-        <v>12.5</v>
+        <v>2.9</v>
       </c>
       <c r="L227">
-        <v>12.8</v>
+        <v>3</v>
       </c>
       <c r="M227">
-        <v>13.4</v>
+        <v>3</v>
       </c>
       <c r="N227">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="228" spans="2:14" x14ac:dyDescent="0.3">
@@ -8508,25 +8516,25 @@
         <v>4</v>
       </c>
       <c r="H228" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I228">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J228">
-        <v>17</v>
+        <v>13.7</v>
       </c>
       <c r="K228">
-        <v>16.5</v>
+        <v>12.5</v>
       </c>
       <c r="L228">
-        <v>18.5</v>
+        <v>12.8</v>
       </c>
       <c r="M228">
-        <v>20</v>
+        <v>13.4</v>
       </c>
       <c r="N228">
-        <v>21.5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="229" spans="2:14" x14ac:dyDescent="0.3">
@@ -8534,28 +8542,28 @@
         <v>67</v>
       </c>
       <c r="G229" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H229" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I229">
-        <v>3.5</v>
+        <v>18</v>
       </c>
       <c r="J229">
-        <v>3.6</v>
+        <v>17</v>
       </c>
       <c r="K229">
-        <v>4.0999999999999996</v>
+        <v>16.5</v>
       </c>
       <c r="L229">
-        <v>4.3</v>
+        <v>18.5</v>
       </c>
       <c r="M229">
-        <v>4.5999999999999996</v>
+        <v>20</v>
       </c>
       <c r="N229">
-        <v>4.9000000000000004</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="230" spans="2:14" x14ac:dyDescent="0.3">
@@ -8566,25 +8574,25 @@
         <v>6</v>
       </c>
       <c r="H230" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I230">
-        <v>12</v>
+        <v>3.5</v>
       </c>
       <c r="J230">
-        <v>13</v>
+        <v>3.6</v>
       </c>
       <c r="K230">
-        <v>12.7</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="L230">
-        <v>12.4</v>
+        <v>4.3</v>
       </c>
       <c r="M230">
-        <v>13.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="N230">
-        <v>17</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="231" spans="2:14" x14ac:dyDescent="0.3">
@@ -8595,25 +8603,25 @@
         <v>6</v>
       </c>
       <c r="H231" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I231">
-        <v>15.5</v>
+        <v>12</v>
       </c>
       <c r="J231">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K231">
-        <v>15.5</v>
+        <v>12.7</v>
       </c>
       <c r="L231">
-        <v>15.5</v>
+        <v>12.4</v>
       </c>
       <c r="M231">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="N231">
-        <v>19.5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="232" spans="2:14" x14ac:dyDescent="0.3">
@@ -8621,28 +8629,28 @@
         <v>67</v>
       </c>
       <c r="G232" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H232" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I232">
-        <v>8.6999999999999993</v>
+        <v>15.5</v>
       </c>
       <c r="J232">
-        <v>9.4</v>
+        <v>16</v>
       </c>
       <c r="K232">
-        <v>11</v>
+        <v>15.5</v>
       </c>
       <c r="L232">
-        <v>11.9</v>
+        <v>15.5</v>
       </c>
       <c r="M232">
-        <v>12.4</v>
+        <v>16.5</v>
       </c>
       <c r="N232">
-        <v>12.4</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="233" spans="2:14" x14ac:dyDescent="0.3">
@@ -8653,25 +8661,25 @@
         <v>5</v>
       </c>
       <c r="H233" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I233">
-        <v>10.6</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="J233">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="K233">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L233">
-        <v>13.5</v>
+        <v>11.9</v>
       </c>
       <c r="M233">
-        <v>14.7</v>
+        <v>12.4</v>
       </c>
       <c r="N233">
-        <v>15</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="234" spans="2:14" x14ac:dyDescent="0.3">
@@ -8682,54 +8690,54 @@
         <v>5</v>
       </c>
       <c r="H234" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I234">
-        <v>14.2</v>
+        <v>10.6</v>
       </c>
       <c r="J234">
-        <v>14</v>
+        <v>10.4</v>
       </c>
       <c r="K234">
-        <v>14.8</v>
+        <v>13</v>
       </c>
       <c r="L234">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="M234">
-        <v>19.5</v>
+        <v>14.7</v>
       </c>
       <c r="N234">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B235" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G235" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H235" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I235">
-        <v>1.9</v>
+        <v>14.2</v>
       </c>
       <c r="J235">
-        <v>1.8</v>
+        <v>14</v>
       </c>
       <c r="K235">
-        <v>1.5</v>
+        <v>14.8</v>
       </c>
       <c r="L235">
-        <v>1.6</v>
+        <v>16.5</v>
       </c>
       <c r="M235">
-        <v>2.2000000000000002</v>
+        <v>19.5</v>
       </c>
       <c r="N235">
-        <v>2.5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="236" spans="2:14" x14ac:dyDescent="0.3">
@@ -8740,25 +8748,25 @@
         <v>3</v>
       </c>
       <c r="H236" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I236">
-        <v>11.5</v>
+        <v>1.9</v>
       </c>
       <c r="J236">
-        <v>11.7</v>
+        <v>1.8</v>
       </c>
       <c r="K236">
-        <v>16</v>
+        <v>1.5</v>
       </c>
       <c r="L236">
-        <v>14.3</v>
+        <v>1.6</v>
       </c>
       <c r="M236">
-        <v>15.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="N236">
-        <v>15.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="237" spans="2:14" x14ac:dyDescent="0.3">
@@ -8769,25 +8777,25 @@
         <v>3</v>
       </c>
       <c r="H237" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I237">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="J237">
-        <v>14.5</v>
+        <v>11.7</v>
       </c>
       <c r="K237">
-        <v>21.5</v>
+        <v>16</v>
       </c>
       <c r="L237">
-        <v>21.8</v>
+        <v>14.3</v>
       </c>
       <c r="M237">
-        <v>22</v>
+        <v>15.5</v>
       </c>
       <c r="N237">
-        <v>23</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="238" spans="2:14" x14ac:dyDescent="0.3">
@@ -8795,28 +8803,28 @@
         <v>68</v>
       </c>
       <c r="G238" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H238" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I238">
-        <v>1.6</v>
+        <v>15</v>
       </c>
       <c r="J238">
-        <v>2</v>
+        <v>14.5</v>
       </c>
       <c r="K238">
-        <v>2.5</v>
+        <v>21.5</v>
       </c>
       <c r="L238">
-        <v>2.6</v>
+        <v>21.8</v>
       </c>
       <c r="M238">
-        <v>2.6</v>
+        <v>22</v>
       </c>
       <c r="N238">
-        <v>2.6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="239" spans="2:14" x14ac:dyDescent="0.3">
@@ -8827,25 +8835,25 @@
         <v>4</v>
       </c>
       <c r="H239" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I239">
-        <v>11.3</v>
+        <v>1.6</v>
       </c>
       <c r="J239">
-        <v>10.3</v>
+        <v>2</v>
       </c>
       <c r="K239">
-        <v>10.5</v>
+        <v>2.5</v>
       </c>
       <c r="L239">
-        <v>9.5</v>
+        <v>2.6</v>
       </c>
       <c r="M239">
-        <v>9.6999999999999993</v>
+        <v>2.6</v>
       </c>
       <c r="N239">
-        <v>10.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="240" spans="2:14" x14ac:dyDescent="0.3">
@@ -8856,25 +8864,25 @@
         <v>4</v>
       </c>
       <c r="H240" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I240">
-        <v>14.5</v>
+        <v>11.3</v>
       </c>
       <c r="J240">
-        <v>13.5</v>
+        <v>10.3</v>
       </c>
       <c r="K240">
-        <v>14</v>
+        <v>10.5</v>
       </c>
       <c r="L240">
-        <v>13.7</v>
+        <v>9.5</v>
       </c>
       <c r="M240">
-        <v>14.3</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="N240">
-        <v>16.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="241" spans="2:14" x14ac:dyDescent="0.3">
@@ -8882,28 +8890,28 @@
         <v>68</v>
       </c>
       <c r="G241" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H241" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I241">
-        <v>2.9</v>
+        <v>14.5</v>
       </c>
       <c r="J241">
-        <v>2.8</v>
+        <v>13.5</v>
       </c>
       <c r="K241">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="L241">
-        <v>3.6</v>
+        <v>13.7</v>
       </c>
       <c r="M241">
-        <v>4</v>
+        <v>14.3</v>
       </c>
       <c r="N241">
-        <v>3.7</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="242" spans="2:14" x14ac:dyDescent="0.3">
@@ -8914,25 +8922,25 @@
         <v>6</v>
       </c>
       <c r="H242" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I242">
-        <v>11.7</v>
+        <v>2.9</v>
       </c>
       <c r="J242">
-        <v>11</v>
+        <v>2.8</v>
       </c>
       <c r="K242">
-        <v>10</v>
+        <v>3.5</v>
       </c>
       <c r="L242">
-        <v>9.6999999999999993</v>
+        <v>3.6</v>
       </c>
       <c r="M242">
-        <v>10.3</v>
+        <v>4</v>
       </c>
       <c r="N242">
-        <v>10.4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="243" spans="2:14" x14ac:dyDescent="0.3">
@@ -8943,25 +8951,25 @@
         <v>6</v>
       </c>
       <c r="H243" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I243">
-        <v>14.5</v>
+        <v>11.7</v>
       </c>
       <c r="J243">
-        <v>13.8</v>
+        <v>11</v>
       </c>
       <c r="K243">
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="L243">
-        <v>12.5</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="M243">
-        <v>13.5</v>
+        <v>10.3</v>
       </c>
       <c r="N243">
-        <v>13.5</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="244" spans="2:14" x14ac:dyDescent="0.3">
@@ -8969,28 +8977,28 @@
         <v>68</v>
       </c>
       <c r="G244" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H244" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I244">
-        <v>8.6999999999999993</v>
+        <v>14.5</v>
       </c>
       <c r="J244">
-        <v>10</v>
+        <v>13.8</v>
       </c>
       <c r="K244">
-        <v>11.9</v>
+        <v>12.5</v>
       </c>
       <c r="L244">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="M244">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="N244">
-        <v>14.8</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="245" spans="2:14" x14ac:dyDescent="0.3">
@@ -9001,25 +9009,25 @@
         <v>5</v>
       </c>
       <c r="H245" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="I245">
-        <v>8.3000000000000007</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="J245">
-        <v>8.6999999999999993</v>
+        <v>10</v>
       </c>
       <c r="K245">
-        <v>8.9</v>
+        <v>11.9</v>
       </c>
       <c r="L245">
-        <v>10.199999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="M245">
-        <v>13.4</v>
+        <v>14</v>
       </c>
       <c r="N245">
-        <v>13.9</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="246" spans="2:14" x14ac:dyDescent="0.3">
@@ -9030,24 +9038,53 @@
         <v>5</v>
       </c>
       <c r="H246" t="s">
+        <v>33</v>
+      </c>
+      <c r="I246">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J246">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="K246">
+        <v>8.9</v>
+      </c>
+      <c r="L246">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="M246">
+        <v>13.4</v>
+      </c>
+      <c r="N246">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="247" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B247" t="s">
+        <v>68</v>
+      </c>
+      <c r="G247" t="s">
+        <v>5</v>
+      </c>
+      <c r="H247" t="s">
         <v>32</v>
       </c>
-      <c r="I246">
+      <c r="I247">
         <v>12</v>
       </c>
-      <c r="J246">
+      <c r="J247">
         <v>12.5</v>
       </c>
-      <c r="K246">
+      <c r="K247">
         <v>12.2</v>
       </c>
-      <c r="L246">
+      <c r="L247">
         <v>13.5</v>
       </c>
-      <c r="M246">
+      <c r="M247">
         <v>17.3</v>
       </c>
-      <c r="N246">
+      <c r="N247">
         <v>18.2</v>
       </c>
     </row>

</xml_diff>